<commit_message>
Add PraNet C1-C4 seed-0 result on C5
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,6 +519,55 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/unet_c1-c4_seed0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PraNet</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://github.com/DengPingFan/PraNet@95f12bd4e32ec954b5069654abae7de9473fd1f5</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>19</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.5796</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.5104</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>MyTrain.py defaults, 19 epochs, last snapshot; Res2Net-50 v1b ImageNet backbone; C5 maps as in MyTest.py (lateral map 2, min-max per image)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/pranet_c1-c4_seed0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Polyp-PVT C1-C4 seed-0 result on C5
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,6 +568,55 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/pranet_c1-c4_seed0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Polyp-PVT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://github.com/DengPingFan/Polyp-PVT@cd71fbf9fcd8c32cc0f33699f4e0186073c64dc4</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>99</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.6442</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.5721000000000001</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Train.py defaults, 99 epochs, last epoch (per-epoch public test-set selection off); PVTv2-B2 ImageNet backbone; C5 maps as in Test.py (P1+P2, min-max per image)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/polyp-pvt_c1-c4_seed0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SAM2-UNet C1-C4 seed-0 result on C5
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AB5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -922,6 +922,128 @@
       <c r="AB4" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/polyp-pvt_c1-c4_seed0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sam2-unet_c1-c4_seed0</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SAM2-UNet</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Visual Intelligence 2026 (arXiv 2024)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://github.com/WZH0120/SAM2-UNet@01598e5e9912ffb23f965ecbebf4d1dfecbaa56e</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>SAM2 Hiera-L, frozen, with adapters</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>SAM2 sam2_hiera_large.pt (Meta, dl.fbaipublicfiles.com)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>352x352</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>horizontal and vertical flip</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 3 maps</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>AdamW, weight decay 5e-4, cosine decay to 1e-7</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="N5" t="n">
+        <v>12</v>
+      </c>
+      <c r="O5" t="n">
+        <v>20</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>last epoch (SAM2-UNet-20.pth)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T5" t="n">
+        <v>208</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>NVIDIA RTX 5000 Ada Generation</t>
+        </is>
+      </c>
+      <c r="W5" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.6584</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.593</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>train.py defaults; C5 maps = first output, min-max per image as in test.py</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/sam2-unet_c1-c4_seed0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add EMCAD C1-C4 seed-0 result on C5
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB5"/>
+  <dimension ref="A1:AB6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1044,6 +1044,128 @@
       <c r="AB5" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/sam2-unet_c1-c4_seed0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>emcad_c1-c4_seed0</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>EMCAD</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://github.com/SLDGroup/EMCAD@26c9c31f731f749b62c5fe83f44376dac75f3aa8</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PVTv2-B2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ImageNet PVTv2-B2 (PVT GitHub release v2, pvt_v2_b2.pth)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>352x352, multi-scale training 0.75/1/1.25</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>rotate up to 90 deg, vertical and horizontal flip (albumentations)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 4 maps and their sum</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>AdamW, weight decay 1e-4, cosine decay to 1e-6, gradient clip 0.5</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="N6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O6" t="n">
+        <v>200</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>last epoch (EMCAD-last.pth); per-epoch val selection off</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T6" t="n">
+        <v>208</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>NVIDIA RTX 5000 Ada Generation</t>
+        </is>
+      </c>
+      <c r="W6" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.6608000000000001</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.5754</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>train_polyp.py defaults, one run of the five its loop trains; C5 inputs from its own OpenCV loader; C5 maps = last output, min-max per image as in test_polyp.py, resized to the true mask size (test_polyp.py swaps height and width)</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/emcad_c1-c4_seed0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add nnU-Net 2d C1-C4 seed-0 result on C5
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB6"/>
+  <dimension ref="A1:AB7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1166,6 +1166,128 @@
       <c r="AB6" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/emcad_c1-c4_seed0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>nnunet-2d_c1-c4_seed0</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>nnU-Net</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Nature Methods 2021</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://github.com/MIC-DKFZ/nnUNet@468cf803df9b267150ae2b6c0c59b8ac84f16227</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>none (U-Net from nnU-Net plans, trained from scratch)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>1024x1536 patches (nnUNetPlans.json; median image 1080x1440, no resampling)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>nnU-Net default (rotation, scaling, noise, blur, brightness, contrast, low resolution, gamma, mirroring)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Dice + cross-entropy, deep supervision</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>SGD Nesterov momentum 0.99, weight decay 3e-5, poly learning-rate decay</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="N7" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>final epoch (checkpoint_final.pth)</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T7" t="n">
+        <v>208</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>NVIDIA RTX 5000 Ada Generation</t>
+        </is>
+      </c>
+      <c r="W7" t="n">
+        <v>12.05</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0.5938</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0.5134</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>9</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>nnU-Net v2.8.1 defaults, 2d, fold all, 1000 epochs x 250 iterations; nnUNetv2_predict defaults (mirroring TTA); labels 0/1 saved as 0/255</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/nnunet-2d_c1-c4_seed0</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1214,6 +1336,23 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Why training was fast: the training set is small, 1,241 single frames (PolypGen C1-C4) at 352x352, and each repo was run with its default number of epochs. Train time per model on one NVIDIA RTX 5000 Ada (32 GB): U-Net 0.28 h (100 epochs x 78 batches of 16), PraNet 0.18 h (19 epochs x 78 batches of 16, each at 3 scales), Polyp-PVT 1.11 h (99 epochs x 78 batches of 16, each at 3 scales). Train time is the Slurm job run time (RunTime, the quantity sacct reports as Elapsed) and includes model loading and the C5 prediction (under a minute). The sacct database was unreachable on 2026-10-14, so these three values were read with scontrol when each job ended; later jobs print their StartTime and RunTime into their logs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Train time of the three newer baselines on the same GPU (Slurm RunTime from the job logs, including C5 prediction): SAM2-UNet 0.35 h (20 epochs, batches of 12 at 352x352), EMCAD 2.52 h (200 epochs x 156 batches of 8, each at 3 scales, about 45 s per epoch), nnU-Net 12.05 h (1000 epochs x 250 iterations of 2 full-resolution 1024x1536 patches, mean epoch time 38 s = 10.6 h, plus planning, preprocessing, checkpointing and its own final validation). nnU-Net takes longest because its default trains 1000 epochs on full-resolution patches; the other models resize frames to 352x352.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add PraNet seed 1-2 and Polyp-PVT+BigAug seed 0 results on C5
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB7"/>
+  <dimension ref="A1:AB10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1288,6 +1288,372 @@
       <c r="AB7" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/nnunet-2d_c1-c4_seed0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>polyp-pvt-bigaug_c1-c4_seed0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Polyp-PVT + BigAug</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>CAAI Artificial Intelligence Research 2023 (Polyp-PVT); IEEE TMI 2020 (BigAug)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://github.com/DengPingFan/Polyp-PVT@cd71fbf9fcd8c32cc0f33699f4e0186073c64dc4</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PVTv2-B2</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ImageNet PVTv2-B2 (pvt_v2_b2.pth from the Polyp-PVT Google Drive; same bytes as the PVT GitHub release)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>352x352, multi-scale training 0.75/1/1.25</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>BigAug image quality (sharpen: unsharp masking strength 10-30; Gaussian blur std 0.25-1.5 px; Gaussian noise std 0.1-1.0) and appearance (brightness shift +-0.1; gamma 0.5-4.5; intensity scale and shift +-0.1), each p 0.5; multi-scale resizing</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 2 maps</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>AdamW, weight decay 1e-4, gradient clip 0.5</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="N8" t="n">
+        <v>16</v>
+      </c>
+      <c r="O8" t="n">
+        <v>99</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>last epoch (99PolypPVT.pth); per-epoch public test-set selection off</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>208</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>NVIDIA RTX 5000 Ada Generation</t>
+        </is>
+      </c>
+      <c r="W8" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0.6296</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0.5498</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>17</v>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Plain Polyp-PVT run plus BigAug image-quality and appearance transforms, each with p 0.5, ranges from the paper; the unsharp-masking blur widths (0.5-1.0 and 0.5 px) and the scale formula x*(1+s) and the clip to [0,1] after each transform are ours; the paper's noise std 0.1-1.0 on [0,1] intensities buries some training frames in noise; spatial BigAug transforms not used; no BigAug at test time</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/polyp-pvt-bigaug_c1-c4_seed0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>pranet_c1-c4_seed1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PraNet</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MICCAI 2020</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://github.com/DengPingFan/PraNet@95f12bd4e32ec954b5069654abae7de9473fd1f5</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Res2Net-50 v1b 26w 4s</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ImageNet Res2Net-50 v1b (res2net50_v1b_26w_4s-3cf99910.pth, official Res2Net URL)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>352x352, multi-scale training 0.75/1/1.25</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>none (multi-scale resizing only)</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 4 maps</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Adam, gradient clip 0.5</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="N9" t="n">
+        <v>16</v>
+      </c>
+      <c r="O9" t="n">
+        <v>19</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>last epoch (PraNet-19.pth)</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T9" t="n">
+        <v>208</v>
+      </c>
+      <c r="U9" t="n">
+        <v>1</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>NVIDIA RTX 5000 Ada Generation</t>
+        </is>
+      </c>
+      <c r="W9" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0.5149</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0.4514</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>11</v>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>MyTrain.py defaults, 19 epochs, last snapshot; Res2Net-50 v1b ImageNet backbone; C5 maps as in MyTest.py (lateral map 2, min-max per image)</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/pranet_c1-c4_seed1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>pranet_c1-c4_seed2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PraNet</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>MICCAI 2020</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://github.com/DengPingFan/PraNet@95f12bd4e32ec954b5069654abae7de9473fd1f5</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Res2Net-50 v1b 26w 4s</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ImageNet Res2Net-50 v1b (res2net50_v1b_26w_4s-3cf99910.pth, official Res2Net URL)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>352x352, multi-scale training 0.75/1/1.25</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>none (multi-scale resizing only)</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 4 maps</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Adam, gradient clip 0.5</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="N10" t="n">
+        <v>16</v>
+      </c>
+      <c r="O10" t="n">
+        <v>19</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>last epoch (PraNet-19.pth)</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T10" t="n">
+        <v>208</v>
+      </c>
+      <c r="U10" t="n">
+        <v>2</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>NVIDIA RTX 5000 Ada Generation</t>
+        </is>
+      </c>
+      <c r="W10" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0.5225</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0.4626</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>46</v>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>MyTrain.py defaults, 19 epochs, last snapshot; Res2Net-50 v1b ImageNet backbone; C5 maps as in MyTest.py (lateral map 2, min-max per image)</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/pranet_c1-c4_seed2</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1353,6 +1719,23 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>Train time of the three newer baselines on the same GPU (Slurm RunTime from the job logs, including C5 prediction): SAM2-UNet 0.35 h (20 epochs, batches of 12 at 352x352), EMCAD 2.52 h (200 epochs x 156 batches of 8, each at 3 scales, about 45 s per epoch), nnU-Net 12.05 h (1000 epochs x 250 iterations of 2 full-resolution 1024x1536 patches, mean epoch time 38 s = 10.6 h, plus planning, preprocessing, checkpointing and its own final validation). nnU-Net takes longest because its default trains 1000 epochs on full-resolution patches; the other models resize frames to 352x352.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PraNet (pranet_c1-c4), seeds 0, 1, 2 on C5: Dice 0.5390 +- 0.0354, IoU 0.4748 +- 0.0313 (mean +- sample standard deviation over the 3 runs)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add U-Net seed 1-2 results on C5
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB10"/>
+  <dimension ref="A1:AB12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1654,6 +1654,250 @@
       <c r="AB10" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/pranet_c1-c4_seed2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>unet_c1-c4_seed1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>U-Net</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MICCAI 2015 (U-Net); encoder from segmentation_models_pytorch</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>segmentation_models_pytorch (pip)@0.5.0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>ResNet-34</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ImageNet ResNet-34 (smp-hub/resnet34.imagenet)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>352x352</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Dice + BCE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="N11" t="n">
+        <v>16</v>
+      </c>
+      <c r="O11" t="n">
+        <v>100</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>last epoch (unet.pth)</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T11" t="n">
+        <v>208</v>
+      </c>
+      <c r="U11" t="n">
+        <v>1</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>NVIDIA RTX 5000 Ada Generation</t>
+        </is>
+      </c>
+      <c r="W11" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0.5219</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0.4457</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>35</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>smp Unet ResNet-34 ImageNet, Dice+BCE, Adam 1e-4, batch 16, 352 px, no augmentation, last epoch; C5 maps = sigmoid (no min-max)</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/unet_c1-c4_seed1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>unet_c1-c4_seed2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>U-Net</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>MICCAI 2015 (U-Net); encoder from segmentation_models_pytorch</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>segmentation_models_pytorch (pip)@0.5.0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ResNet-34</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>ImageNet ResNet-34 (smp-hub/resnet34.imagenet)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>352x352</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Dice + BCE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="N12" t="n">
+        <v>16</v>
+      </c>
+      <c r="O12" t="n">
+        <v>100</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>last epoch (unet.pth)</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R12" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>208</v>
+      </c>
+      <c r="U12" t="n">
+        <v>2</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>NVIDIA RTX 5000 Ada Generation</t>
+        </is>
+      </c>
+      <c r="W12" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0.5412</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0.4612</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>35</v>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>smp Unet ResNet-34 ImageNet, Dice+BCE, Adam 1e-4, batch 16, 352 px, no augmentation, last epoch; C5 maps = sigmoid (no min-max)</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/unet_c1-c4_seed2</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1736,6 +1980,23 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>PraNet (pranet_c1-c4), seeds 0, 1, 2 on C5: Dice 0.5390 +- 0.0354, IoU 0.4748 +- 0.0313 (mean +- sample standard deviation over the 3 runs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>U-Net (unet_c1-c4), seeds 0, 1, 2 on C5: Dice 0.5100 +- 0.0386, IoU 0.4383 +- 0.0273 (mean +- sample standard deviation over the 3 runs)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SAM2-UNet seed 1 result on C5
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AB13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1898,6 +1898,128 @@
       <c r="AB12" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/unet_c1-c4_seed2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sam2-unet_c1-c4_seed1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SAM2-UNet</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Visual Intelligence 2026 (arXiv 2024)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://github.com/WZH0120/SAM2-UNet@01598e5e9912ffb23f965ecbebf4d1dfecbaa56e</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>SAM2 Hiera-L, frozen, with adapters</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>SAM2 sam2_hiera_large.pt (Meta, dl.fbaipublicfiles.com)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>352x352</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>horizontal and vertical flip</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 3 maps</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>AdamW, weight decay 5e-4, cosine decay to 1e-7</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="N13" t="n">
+        <v>12</v>
+      </c>
+      <c r="O13" t="n">
+        <v>20</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>last epoch (SAM2-UNet-20.pth)</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R13" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T13" t="n">
+        <v>208</v>
+      </c>
+      <c r="U13" t="n">
+        <v>1</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>NVIDIA RTX 5000 Ada Generation</t>
+        </is>
+      </c>
+      <c r="W13" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0.6679</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0.5952</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>train.py defaults; C5 maps = first output, min-max per image as in test.py</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/sam2-unet_c1-c4_seed1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SAM2-UNet seed 2 result on C5
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB13"/>
+  <dimension ref="A1:AB14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2020,6 +2020,128 @@
       <c r="AB13" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/sam2-unet_c1-c4_seed1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>sam2-unet_c1-c4_seed2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SAM2-UNet</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Visual Intelligence 2026 (arXiv 2024)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://github.com/WZH0120/SAM2-UNet@01598e5e9912ffb23f965ecbebf4d1dfecbaa56e</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>SAM2 Hiera-L, frozen, with adapters</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>SAM2 sam2_hiera_large.pt (Meta, dl.fbaipublicfiles.com)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>352x352</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>horizontal and vertical flip</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 3 maps</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>AdamW, weight decay 5e-4, cosine decay to 1e-7</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="N14" t="n">
+        <v>12</v>
+      </c>
+      <c r="O14" t="n">
+        <v>20</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>last epoch (SAM2-UNet-20.pth)</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R14" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T14" t="n">
+        <v>208</v>
+      </c>
+      <c r="U14" t="n">
+        <v>2</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>NVIDIA RTX 5000 Ada Generation</t>
+        </is>
+      </c>
+      <c r="W14" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0.6496</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0.5776</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>train.py defaults; C5 maps = first output, min-max per image as in test.py</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/sam2-unet_c1-c4_seed2</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2119,6 +2241,23 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>U-Net (unet_c1-c4), seeds 0, 1, 2 on C5: Dice 0.5100 +- 0.0386, IoU 0.4383 +- 0.0273 (mean +- sample standard deviation over the 3 runs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SAM2-UNet (sam2-unet_c1-c4), seeds 0, 1, 2 on C5: Dice 0.6586 +- 0.0092, IoU 0.5886 +- 0.0096 (mean +- sample standard deviation over the 3 runs)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Polyp-PVT seed 1 (PC)
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB14"/>
+  <dimension ref="A1:AB15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2142,6 +2142,128 @@
       <c r="AB14" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/sam2-unet_c1-c4_seed2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>polyp-pvt_c1-c4_seed1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Polyp-PVT</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CAAI Artificial Intelligence Research 2023</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://github.com/DengPingFan/Polyp-PVT@cd71fbf9fcd8c32cc0f33699f4e0186073c64dc4</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>PVTv2-B2</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>ImageNet PVTv2-B2 (pvt_v2_b2.pth from the Polyp-PVT Google Drive; same bytes as the PVT GitHub release)</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>352x352, multi-scale training 0.75/1/1.25</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>none (Train.py default --augmentation False; multi-scale resizing only)</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 2 maps</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>AdamW, weight decay 1e-4, gradient clip 0.5</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="N15" t="n">
+        <v>16</v>
+      </c>
+      <c r="O15" t="n">
+        <v>99</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>last epoch (99PolypPVT.pth); per-epoch public test-set selection off</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R15" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>208</v>
+      </c>
+      <c r="U15" t="n">
+        <v>1</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 5060 Ti</t>
+        </is>
+      </c>
+      <c r="W15" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="X15" t="n">
+        <v>0.6395999999999999</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>0.5691000000000001</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>36</v>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>Train.py defaults, 99 epochs, last epoch (per-epoch public test-set selection off); PVTv2-B2 ImageNet backbone; C5 maps as in Test.py (P1+P2, min-max per image); seed 0 ran on RTX 5000 Ada (HPC)</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/polyp-pvt_c1-c4_seed1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Polyp-PVT seed 2 (PC) and the 3-seed note
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB15"/>
+  <dimension ref="A1:AB16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2264,6 +2264,128 @@
       <c r="AB15" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/polyp-pvt_c1-c4_seed1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>polyp-pvt_c1-c4_seed2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Polyp-PVT</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CAAI Artificial Intelligence Research 2023</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://github.com/DengPingFan/Polyp-PVT@cd71fbf9fcd8c32cc0f33699f4e0186073c64dc4</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>PVTv2-B2</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ImageNet PVTv2-B2 (pvt_v2_b2.pth from the Polyp-PVT Google Drive; same bytes as the PVT GitHub release)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>352x352, multi-scale training 0.75/1/1.25</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>none (Train.py default --augmentation False; multi-scale resizing only)</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 2 maps</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>AdamW, weight decay 1e-4, gradient clip 0.5</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="N16" t="n">
+        <v>16</v>
+      </c>
+      <c r="O16" t="n">
+        <v>99</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>last epoch (99PolypPVT.pth); per-epoch public test-set selection off</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R16" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T16" t="n">
+        <v>208</v>
+      </c>
+      <c r="U16" t="n">
+        <v>2</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 5060 Ti</t>
+        </is>
+      </c>
+      <c r="W16" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0.6086</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0.5295</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>Train.py defaults, 99 epochs, last epoch (per-epoch public test-set selection off); PVTv2-B2 ImageNet backbone; C5 maps as in Test.py (P1+P2, min-max per image); seed 0 ran on RTX 5000 Ada (HPC)</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/polyp-pvt_c1-c4_seed2</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2380,6 +2502,23 @@
       <c r="C6" t="inlineStr">
         <is>
           <t>SAM2-UNet (sam2-unet_c1-c4), seeds 0, 1, 2 on C5: Dice 0.6586 +- 0.0092, IoU 0.5886 +- 0.0096 (mean +- sample standard deviation over the 3 runs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Polyp-PVT (polyp-pvt_c1-c4), seeds 0, 1, 2 on C5: Dice 0.6308 +- 0.0194, IoU 0.5569 +- 0.0238 (mean +- sample standard deviation over the 3 runs)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Polyp-PVT + BigAug seed 1 (PC)
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB16"/>
+  <dimension ref="A1:AB17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2386,6 +2386,128 @@
       <c r="AB16" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/polyp-pvt_c1-c4_seed2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>polyp-pvt-bigaug_c1-c4_seed1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Polyp-PVT + BigAug</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CAAI Artificial Intelligence Research 2023 (Polyp-PVT); IEEE TMI 2020 (BigAug)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://github.com/DengPingFan/Polyp-PVT@cd71fbf9fcd8c32cc0f33699f4e0186073c64dc4</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>PVTv2-B2</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>ImageNet PVTv2-B2 (pvt_v2_b2.pth from the Polyp-PVT Google Drive; same bytes as the PVT GitHub release)</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>352x352, multi-scale training 0.75/1/1.25</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>BigAug image quality (sharpen: unsharp masking strength 10-30; Gaussian blur std 0.25-1.5 px; Gaussian noise std 0.1-1.0) and appearance (brightness shift +-0.1; gamma 0.5-4.5; intensity scale and shift +-0.1), each p 0.5; multi-scale resizing</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 2 maps</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>AdamW, weight decay 1e-4, gradient clip 0.5</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="N17" t="n">
+        <v>16</v>
+      </c>
+      <c r="O17" t="n">
+        <v>99</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>last epoch (99PolypPVT.pth); per-epoch public test-set selection off</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R17" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>208</v>
+      </c>
+      <c r="U17" t="n">
+        <v>1</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 5060 Ti</t>
+        </is>
+      </c>
+      <c r="W17" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0.6703</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0.5903</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>19</v>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>Plain Polyp-PVT run plus BigAug image-quality and appearance transforms, each with p 0.5, ranges from the paper; the unsharp-masking blur widths (0.5-1.0 and 0.5 px) and the scale formula x*(1+s) and the clip to [0,1] after each transform are ours; the paper's noise std 0.1-1.0 on [0,1] intensities buries some training frames in noise; spatial BigAug transforms not used; no BigAug at test time; seed 0 ran on RTX 5000 Ada (HPC)</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/polyp-pvt-bigaug_c1-c4_seed1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Polyp-PVT + BigAug seed 2 (PC) and the 3-seed note
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB17"/>
+  <dimension ref="A1:AB18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2508,6 +2508,128 @@
       <c r="AB17" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/polyp-pvt-bigaug_c1-c4_seed1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>polyp-pvt-bigaug_c1-c4_seed2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Polyp-PVT + BigAug</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CAAI Artificial Intelligence Research 2023 (Polyp-PVT); IEEE TMI 2020 (BigAug)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://github.com/DengPingFan/Polyp-PVT@cd71fbf9fcd8c32cc0f33699f4e0186073c64dc4</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>PVTv2-B2</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ImageNet PVTv2-B2 (pvt_v2_b2.pth from the Polyp-PVT Google Drive; same bytes as the PVT GitHub release)</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>352x352, multi-scale training 0.75/1/1.25</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>BigAug image quality (sharpen: unsharp masking strength 10-30; Gaussian blur std 0.25-1.5 px; Gaussian noise std 0.1-1.0) and appearance (brightness shift +-0.1; gamma 0.5-4.5; intensity scale and shift +-0.1), each p 0.5; multi-scale resizing</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 2 maps</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>AdamW, weight decay 1e-4, gradient clip 0.5</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="N18" t="n">
+        <v>16</v>
+      </c>
+      <c r="O18" t="n">
+        <v>99</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>last epoch (99PolypPVT.pth); per-epoch public test-set selection off</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R18" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T18" t="n">
+        <v>208</v>
+      </c>
+      <c r="U18" t="n">
+        <v>2</v>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 5060 Ti</t>
+        </is>
+      </c>
+      <c r="W18" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="X18" t="n">
+        <v>0.6478</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0.5728</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>33</v>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>Plain Polyp-PVT run plus BigAug image-quality and appearance transforms, each with p 0.5, ranges from the paper; the unsharp-masking blur widths (0.5-1.0 and 0.5 px) and the scale formula x*(1+s) and the clip to [0,1] after each transform are ours; the paper's noise std 0.1-1.0 on [0,1] intensities buries some training frames in noise; spatial BigAug transforms not used; no BigAug at test time; seed 0 ran on RTX 5000 Ada (HPC)</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/polyp-pvt-bigaug_c1-c4_seed2</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2641,6 +2763,23 @@
       <c r="C7" t="inlineStr">
         <is>
           <t>Polyp-PVT (polyp-pvt_c1-c4), seeds 0, 1, 2 on C5: Dice 0.6308 +- 0.0194, IoU 0.5569 +- 0.0238 (mean +- sample standard deviation over the 3 runs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Polyp-PVT + BigAug (polyp-pvt-bigaug_c1-c4), seeds 0, 1, 2 on C5: Dice 0.6492 +- 0.0204, IoU 0.5710 +- 0.0203 (mean +- sample standard deviation over the 3 runs)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add EMCAD seed 1 (PC)
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB18"/>
+  <dimension ref="A1:AB19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2630,6 +2630,128 @@
       <c r="AB18" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/polyp-pvt-bigaug_c1-c4_seed2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>emcad_c1-c4_seed1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EMCAD</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://github.com/SLDGroup/EMCAD@26c9c31f731f749b62c5fe83f44376dac75f3aa8</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>PVTv2-B2</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ImageNet PVTv2-B2 (PVT GitHub release v2, pvt_v2_b2.pth)</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>352x352, multi-scale training 0.75/1/1.25</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>rotate up to 90 deg, vertical and horizontal flip (albumentations)</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 4 maps and their sum</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>AdamW, weight decay 1e-4, cosine decay to 1e-6, gradient clip 0.5</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="N19" t="n">
+        <v>8</v>
+      </c>
+      <c r="O19" t="n">
+        <v>200</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>last epoch (EMCAD-last.pth); per-epoch val selection off</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R19" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T19" t="n">
+        <v>208</v>
+      </c>
+      <c r="U19" t="n">
+        <v>1</v>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 5060 Ti</t>
+        </is>
+      </c>
+      <c r="W19" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="X19" t="n">
+        <v>0.6737</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>0.588</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>train_polyp.py defaults, one run of the five its loop trains; C5 inputs from its own OpenCV loader; C5 maps = last output, min-max per image as in test_polyp.py, resized to the true mask size (test_polyp.py swaps height and width); seed 0 ran on RTX 5000 Ada (HPC)</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/emcad_c1-c4_seed1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add EMCAD seed 2 (PC) and the 3-seed note
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB19"/>
+  <dimension ref="A1:AB20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2752,6 +2752,128 @@
       <c r="AB19" t="inlineStr">
         <is>
           <t>/l/users/mohamed.abdalla/medai/outputs/emcad_c1-c4_seed1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>emcad_c1-c4_seed2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EMCAD</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://github.com/SLDGroup/EMCAD@26c9c31f731f749b62c5fe83f44376dac75f3aa8</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>PVTv2-B2</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ImageNet PVTv2-B2 (PVT GitHub release v2, pvt_v2_b2.pth)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>352x352, multi-scale training 0.75/1/1.25</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>rotate up to 90 deg, vertical and horizontal flip (albumentations)</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>structure loss (weighted BCE + weighted IoU) on 4 maps and their sum</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>AdamW, weight decay 1e-4, cosine decay to 1e-6, gradient clip 0.5</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="N20" t="n">
+        <v>8</v>
+      </c>
+      <c r="O20" t="n">
+        <v>200</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>last epoch (EMCAD-last.pth); per-epoch val selection off</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>C1-C4</t>
+        </is>
+      </c>
+      <c r="R20" t="n">
+        <v>1241</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="T20" t="n">
+        <v>208</v>
+      </c>
+      <c r="U20" t="n">
+        <v>2</v>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 5060 Ti</t>
+        </is>
+      </c>
+      <c r="W20" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="X20" t="n">
+        <v>0.6582</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>0.5713</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>train_polyp.py defaults, one run of the five its loop trains; C5 inputs from its own OpenCV loader; C5 maps = last output, min-max per image as in test_polyp.py, resized to the true mask size (test_polyp.py swaps height and width); seed 0 ran on RTX 5000 Ada (HPC)</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>/l/users/mohamed.abdalla/medai/outputs/emcad_c1-c4_seed2</t>
         </is>
       </c>
     </row>
@@ -2766,7 +2888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2902,6 +3024,23 @@
       <c r="C8" t="inlineStr">
         <is>
           <t>Polyp-PVT + BigAug (polyp-pvt-bigaug_c1-c4), seeds 0, 1, 2 on C5: Dice 0.6492 +- 0.0204, IoU 0.5710 +- 0.0203 (mean +- sample standard deviation over the 3 runs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mohamed Abdalla</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>EMCAD (emcad_c1-c4), seeds 0, 1, 2 on C5: Dice 0.6642 +- 0.0083, IoU 0.5782 +- 0.0087 (mean +- sample standard deviation over the 3 runs)</t>
         </is>
       </c>
     </row>

</xml_diff>